<commit_message>
feat: end a tiny table at the first blank row
A tiny sheet used to skip blank rows and keep reading. The field area now
stops at the first blank row, so anything written below the gap is ignored
even when it still looks like fields. This is the rule base sheets already
follow (an empty row 9 means "no file", the first empty data row ends the
table).

- a blank row 6 leaves the table with no field at all -> no lua file
- example: 03_tiny_config.xlsx drops its middle blank row so the happy path
  keeps exporting all fields (output byte-identical to before), and
  04_edge_cases.xlsx gains EarlyStop (stops at the gap) and NoFirstRow
  (a blank row 6 -> no file)
- README / README.zh-CN: document the rule and the two new example sheets
</commit_message>
<xml_diff>
--- a/example/en/import/03_tiny_config.xlsx
+++ b/example/en/import/03_tiny_config.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -651,57 +651,57 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
-        </is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Event rate</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>activity_rate</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Event rate</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>activity_rate</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Notice</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
           <t>notice</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Welcome!</t>
         </is>

</xml_diff>